<commit_message>
Update purchasing sheet with vendor, cash/credit, account fields and Zoho entries summary
</commit_message>
<xml_diff>
--- a/purchasing/Kashif_Purchasing_Sheet.xlsx
+++ b/purchasing/Kashif_Purchasing_Sheet.xlsx
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="DD-MMM-YYYY"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,24 +33,18 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="15"/>
+      <sz val="14"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00555555"/>
+      <color rgb="00444444"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001A3A6B"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="008B4513"/>
       <sz val="12"/>
     </font>
     <font>
@@ -71,7 +65,7 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="00666666"/>
+      <color rgb="00555555"/>
       <sz val="11"/>
     </font>
     <font>
@@ -94,24 +88,49 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <color rgb="00333333"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E6B3A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="13"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="001A3A6B"/>
-      <sz val="13"/>
+      <color rgb="001E6B3A"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <i val="1"/>
+      <color rgb="008B0000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="008B0000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00333333"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <color rgb="00555555"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -150,7 +169,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
+        <fgColor rgb="00EAD1DC"/>
       </patternFill>
     </fill>
     <fill>
@@ -160,7 +179,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFDE7"/>
+        <fgColor rgb="00F5F5F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5E6EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDEDEC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007B3F00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF8F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF0E0"/>
       </patternFill>
     </fill>
   </fills>
@@ -174,23 +218,23 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00AAAAAA"/>
+        <color rgb="00BBBBBB"/>
       </left>
       <right style="thin">
-        <color rgb="00AAAAAA"/>
+        <color rgb="00BBBBBB"/>
       </right>
       <top style="thin">
-        <color rgb="00AAAAAA"/>
+        <color rgb="00BBBBBB"/>
       </top>
       <bottom style="thin">
-        <color rgb="00AAAAAA"/>
+        <color rgb="00BBBBBB"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -201,59 +245,101 @@
     <xf numFmtId="164" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="12" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="16" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="12" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="13" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -620,26 +706,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:H54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ZIDANE CORPORATION  —  PURCHASING SHEET</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="2" t="inlineStr"/>
+          <t>ZIDANE CORPORATION  ·  PURCHASING SHEET</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
           <t>DATE</t>
@@ -657,13 +744,20 @@
           <t>ADVANCE GIVEN (PKR)</t>
         </is>
       </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>PAID FROM (ACCOUNT)</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="B3" s="3" t="n"/>
       <c r="D3" s="4" t="n"/>
       <c r="F3" s="5" t="n"/>
-    </row>
-    <row r="4" ht="6" customHeight="1"/>
+      <c r="G3" s="4" t="n"/>
+    </row>
+    <row r="4" ht="5" customHeight="1"/>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
@@ -693,6 +787,16 @@
       <c r="F5" s="6" t="inlineStr">
         <is>
           <t>AMOUNT (PKR)</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>VENDOR / SUPPLIER</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>CASH / CREDIT</t>
         </is>
       </c>
     </row>
@@ -718,22 +822,28 @@
         <f>IF(E6="","",D6*E6)</f>
         <v/>
       </c>
+      <c r="G6" s="13" t="n"/>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="13" t="n">
+      <c r="A7" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="16" t="inlineStr">
         <is>
           <t>AIR FRESHNER ROOM SPRAY 300ML TOPIC BRAND</t>
         </is>
       </c>
-      <c r="C7" s="15" t="inlineStr">
+      <c r="C7" s="17" t="inlineStr">
         <is>
           <t>PCS</t>
         </is>
       </c>
-      <c r="D7" s="16" t="n">
+      <c r="D7" s="18" t="n">
         <v>96</v>
       </c>
       <c r="E7" s="11" t="n"/>
@@ -741,6 +851,12 @@
         <f>IF(E7="","",D7*E7)</f>
         <v/>
       </c>
+      <c r="G7" s="19" t="n"/>
+      <c r="H7" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="7" t="n">
@@ -764,22 +880,28 @@
         <f>IF(E8="","",D8*E8)</f>
         <v/>
       </c>
+      <c r="G8" s="13" t="n"/>
+      <c r="H8" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="13" t="n">
+      <c r="A9" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>BROOM HARD</t>
         </is>
       </c>
-      <c r="C9" s="15" t="inlineStr">
+      <c r="C9" s="17" t="inlineStr">
         <is>
           <t>PCS</t>
         </is>
       </c>
-      <c r="D9" s="16" t="n">
+      <c r="D9" s="18" t="n">
         <v>200</v>
       </c>
       <c r="E9" s="11" t="n"/>
@@ -787,6 +909,12 @@
         <f>IF(E9="","",D9*E9)</f>
         <v/>
       </c>
+      <c r="G9" s="19" t="n"/>
+      <c r="H9" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="7" t="n">
@@ -810,22 +938,28 @@
         <f>IF(E10="","",D10*E10)</f>
         <v/>
       </c>
+      <c r="G10" s="13" t="n"/>
+      <c r="H10" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="13" t="n">
+      <c r="A11" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B11" s="16" t="inlineStr">
         <is>
           <t>CHINA BRUSH</t>
         </is>
       </c>
-      <c r="C11" s="15" t="inlineStr">
+      <c r="C11" s="17" t="inlineStr">
         <is>
           <t>PCS</t>
         </is>
       </c>
-      <c r="D11" s="16" t="n">
+      <c r="D11" s="18" t="n">
         <v>130</v>
       </c>
       <c r="E11" s="11" t="n"/>
@@ -833,6 +967,12 @@
         <f>IF(E11="","",D11*E11)</f>
         <v/>
       </c>
+      <c r="G11" s="19" t="n"/>
+      <c r="H11" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="7" t="n">
@@ -856,22 +996,28 @@
         <f>IF(E12="","",D12*E12)</f>
         <v/>
       </c>
+      <c r="G12" s="13" t="n"/>
+      <c r="H12" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="13" t="n">
+      <c r="A13" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="B13" s="14" t="inlineStr">
+      <c r="B13" s="16" t="inlineStr">
         <is>
           <t>DUSTER FABRIC</t>
         </is>
       </c>
-      <c r="C13" s="15" t="inlineStr">
+      <c r="C13" s="17" t="inlineStr">
         <is>
           <t>PCS</t>
         </is>
       </c>
-      <c r="D13" s="16" t="n">
+      <c r="D13" s="18" t="n">
         <v>100</v>
       </c>
       <c r="E13" s="11" t="n"/>
@@ -879,6 +1025,12 @@
         <f>IF(E13="","",D13*E13)</f>
         <v/>
       </c>
+      <c r="G13" s="19" t="n"/>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="7" t="n">
@@ -902,22 +1054,28 @@
         <f>IF(E14="","",D14*E14)</f>
         <v/>
       </c>
+      <c r="G14" s="13" t="n"/>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="13" t="n">
+      <c r="A15" s="15" t="n">
         <v>10</v>
       </c>
-      <c r="B15" s="14" t="inlineStr">
+      <c r="B15" s="16" t="inlineStr">
         <is>
           <t>HAND BRUSH</t>
         </is>
       </c>
-      <c r="C15" s="15" t="inlineStr">
+      <c r="C15" s="17" t="inlineStr">
         <is>
           <t>PCS</t>
         </is>
       </c>
-      <c r="D15" s="16" t="n">
+      <c r="D15" s="18" t="n">
         <v>24</v>
       </c>
       <c r="E15" s="11" t="n"/>
@@ -925,6 +1083,12 @@
         <f>IF(E15="","",D15*E15)</f>
         <v/>
       </c>
+      <c r="G15" s="19" t="n"/>
+      <c r="H15" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="7" t="n">
@@ -948,22 +1112,28 @@
         <f>IF(E16="","",D16*E16)</f>
         <v/>
       </c>
+      <c r="G16" s="13" t="n"/>
+      <c r="H16" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="13" t="n">
+      <c r="A17" s="15" t="n">
         <v>12</v>
       </c>
-      <c r="B17" s="14" t="inlineStr">
+      <c r="B17" s="16" t="inlineStr">
         <is>
           <t>LEMON MAX BAR 285 GRAMS</t>
         </is>
       </c>
-      <c r="C17" s="15" t="inlineStr">
+      <c r="C17" s="17" t="inlineStr">
         <is>
           <t>PCS</t>
         </is>
       </c>
-      <c r="D17" s="16" t="n">
+      <c r="D17" s="18" t="n">
         <v>48</v>
       </c>
       <c r="E17" s="11" t="n"/>
@@ -971,6 +1141,12 @@
         <f>IF(E17="","",D17*E17)</f>
         <v/>
       </c>
+      <c r="G17" s="19" t="n"/>
+      <c r="H17" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="7" t="n">
@@ -994,22 +1170,28 @@
         <f>IF(E18="","",D18*E18)</f>
         <v/>
       </c>
+      <c r="G18" s="13" t="n"/>
+      <c r="H18" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="13" t="n">
+      <c r="A19" s="15" t="n">
         <v>14</v>
       </c>
-      <c r="B19" s="14" t="inlineStr">
+      <c r="B19" s="16" t="inlineStr">
         <is>
           <t>MOP BIG 18 X 18 WOODEN</t>
         </is>
       </c>
-      <c r="C19" s="15" t="inlineStr">
+      <c r="C19" s="17" t="inlineStr">
         <is>
           <t>PCS</t>
         </is>
       </c>
-      <c r="D19" s="16" t="n">
+      <c r="D19" s="18" t="n">
         <v>100</v>
       </c>
       <c r="E19" s="11" t="n"/>
@@ -1017,6 +1199,12 @@
         <f>IF(E19="","",D19*E19)</f>
         <v/>
       </c>
+      <c r="G19" s="19" t="n"/>
+      <c r="H19" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="7" t="n">
@@ -1040,22 +1228,28 @@
         <f>IF(E20="","",D20*E20)</f>
         <v/>
       </c>
+      <c r="G20" s="13" t="n"/>
+      <c r="H20" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="13" t="n">
+      <c r="A21" s="15" t="n">
         <v>16</v>
       </c>
-      <c r="B21" s="14" t="inlineStr">
+      <c r="B21" s="16" t="inlineStr">
         <is>
           <t>MOP STICK</t>
         </is>
       </c>
-      <c r="C21" s="15" t="inlineStr">
+      <c r="C21" s="17" t="inlineStr">
         <is>
           <t>PCS</t>
         </is>
       </c>
-      <c r="D21" s="16" t="n">
+      <c r="D21" s="18" t="n">
         <v>48</v>
       </c>
       <c r="E21" s="11" t="n"/>
@@ -1063,6 +1257,12 @@
         <f>IF(E21="","",D21*E21)</f>
         <v/>
       </c>
+      <c r="G21" s="19" t="n"/>
+      <c r="H21" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="7" t="n">
@@ -1086,22 +1286,28 @@
         <f>IF(E22="","",D22*E22)</f>
         <v/>
       </c>
+      <c r="G22" s="13" t="n"/>
+      <c r="H22" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="13" t="n">
+      <c r="A23" s="15" t="n">
         <v>18</v>
       </c>
-      <c r="B23" s="14" t="inlineStr">
+      <c r="B23" s="16" t="inlineStr">
         <is>
           <t>ROOMI BOX</t>
         </is>
       </c>
-      <c r="C23" s="15" t="inlineStr">
+      <c r="C23" s="17" t="inlineStr">
         <is>
           <t>CTN</t>
         </is>
       </c>
-      <c r="D23" s="16" t="n">
+      <c r="D23" s="18" t="n">
         <v>1</v>
       </c>
       <c r="E23" s="11" t="n"/>
@@ -1109,6 +1315,12 @@
         <f>IF(E23="","",D23*E23)</f>
         <v/>
       </c>
+      <c r="G23" s="19" t="n"/>
+      <c r="H23" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="7" t="n">
@@ -1132,22 +1344,28 @@
         <f>IF(E24="","",D24*E24)</f>
         <v/>
       </c>
+      <c r="G24" s="13" t="n"/>
+      <c r="H24" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="13" t="n">
+      <c r="A25" s="15" t="n">
         <v>20</v>
       </c>
-      <c r="B25" s="14" t="inlineStr">
+      <c r="B25" s="16" t="inlineStr">
         <is>
           <t>SCRAPER PLASTIC SUPRI</t>
         </is>
       </c>
-      <c r="C25" s="15" t="inlineStr">
+      <c r="C25" s="17" t="inlineStr">
         <is>
           <t>PCS</t>
         </is>
       </c>
-      <c r="D25" s="16" t="n">
+      <c r="D25" s="18" t="n">
         <v>48</v>
       </c>
       <c r="E25" s="11" t="n"/>
@@ -1155,6 +1373,12 @@
         <f>IF(E25="","",D25*E25)</f>
         <v/>
       </c>
+      <c r="G25" s="19" t="n"/>
+      <c r="H25" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="7" t="n">
@@ -1178,22 +1402,28 @@
         <f>IF(E26="","",D26*E26)</f>
         <v/>
       </c>
+      <c r="G26" s="13" t="n"/>
+      <c r="H26" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="13" t="n">
+      <c r="A27" s="15" t="n">
         <v>22</v>
       </c>
-      <c r="B27" s="14" t="inlineStr">
+      <c r="B27" s="16" t="inlineStr">
         <is>
           <t>TILE WASH SWEEP LOCAL 30KG</t>
         </is>
       </c>
-      <c r="C27" s="15" t="inlineStr">
+      <c r="C27" s="17" t="inlineStr">
         <is>
           <t>CAN</t>
         </is>
       </c>
-      <c r="D27" s="16" t="n">
+      <c r="D27" s="18" t="n">
         <v>9</v>
       </c>
       <c r="E27" s="11" t="n"/>
@@ -1201,6 +1431,12 @@
         <f>IF(E27="","",D27*E27)</f>
         <v/>
       </c>
+      <c r="G27" s="19" t="n"/>
+      <c r="H27" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="7" t="n">
@@ -1224,22 +1460,28 @@
         <f>IF(E28="","",D28*E28)</f>
         <v/>
       </c>
+      <c r="G28" s="13" t="n"/>
+      <c r="H28" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="13" t="n">
+      <c r="A29" s="15" t="n">
         <v>24</v>
       </c>
-      <c r="B29" s="14" t="inlineStr">
+      <c r="B29" s="16" t="inlineStr">
         <is>
           <t>TISSUE PAPER ROLL</t>
         </is>
       </c>
-      <c r="C29" s="15" t="inlineStr">
+      <c r="C29" s="17" t="inlineStr">
         <is>
           <t>PCS</t>
         </is>
       </c>
-      <c r="D29" s="16" t="n">
+      <c r="D29" s="18" t="n">
         <v>200</v>
       </c>
       <c r="E29" s="11" t="n"/>
@@ -1247,6 +1489,12 @@
         <f>IF(E29="","",D29*E29)</f>
         <v/>
       </c>
+      <c r="G29" s="19" t="n"/>
+      <c r="H29" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="7" t="n">
@@ -1270,22 +1518,28 @@
         <f>IF(E30="","",D30*E30)</f>
         <v/>
       </c>
+      <c r="G30" s="13" t="n"/>
+      <c r="H30" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="13" t="n">
+      <c r="A31" s="15" t="n">
         <v>26</v>
       </c>
-      <c r="B31" s="14" t="inlineStr">
+      <c r="B31" s="16" t="inlineStr">
         <is>
           <t>CERAMIC FIBRE ROPE 10MM DIA X 30M TEMP 150-200C</t>
         </is>
       </c>
-      <c r="C31" s="15" t="inlineStr">
+      <c r="C31" s="17" t="inlineStr">
         <is>
           <t>PCS</t>
         </is>
       </c>
-      <c r="D31" s="16" t="n">
+      <c r="D31" s="18" t="n">
         <v>4</v>
       </c>
       <c r="E31" s="11" t="n"/>
@@ -1293,6 +1547,12 @@
         <f>IF(E31="","",D31*E31)</f>
         <v/>
       </c>
+      <c r="G31" s="19" t="n"/>
+      <c r="H31" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="7" t="n">
@@ -1316,22 +1576,28 @@
         <f>IF(E32="","",D32*E32)</f>
         <v/>
       </c>
+      <c r="G32" s="13" t="n"/>
+      <c r="H32" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="13" t="n">
+      <c r="A33" s="15" t="n">
         <v>28</v>
       </c>
-      <c r="B33" s="14" t="inlineStr">
+      <c r="B33" s="16" t="inlineStr">
         <is>
           <t>CERAMIC PLATES WHITE 8INCH</t>
         </is>
       </c>
-      <c r="C33" s="15" t="inlineStr">
+      <c r="C33" s="17" t="inlineStr">
         <is>
           <t>PCS</t>
         </is>
       </c>
-      <c r="D33" s="16" t="n">
+      <c r="D33" s="18" t="n">
         <v>12</v>
       </c>
       <c r="E33" s="11" t="n"/>
@@ -1339,6 +1605,12 @@
         <f>IF(E33="","",D33*E33)</f>
         <v/>
       </c>
+      <c r="G33" s="19" t="n"/>
+      <c r="H33" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="7" t="n">
@@ -1362,22 +1634,28 @@
         <f>IF(E34="","",D34*E34)</f>
         <v/>
       </c>
+      <c r="G34" s="13" t="n"/>
+      <c r="H34" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="13" t="n">
+      <c r="A35" s="15" t="n">
         <v>30</v>
       </c>
-      <c r="B35" s="14" t="inlineStr">
+      <c r="B35" s="16" t="inlineStr">
         <is>
           <t>TABLE SPOON STAINLESS STEEL</t>
         </is>
       </c>
-      <c r="C35" s="15" t="inlineStr">
+      <c r="C35" s="17" t="inlineStr">
         <is>
           <t>DZN</t>
         </is>
       </c>
-      <c r="D35" s="16" t="n">
+      <c r="D35" s="18" t="n">
         <v>2</v>
       </c>
       <c r="E35" s="11" t="n"/>
@@ -1385,6 +1663,12 @@
         <f>IF(E35="","",D35*E35)</f>
         <v/>
       </c>
+      <c r="G35" s="19" t="n"/>
+      <c r="H35" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="7" t="n">
@@ -1408,22 +1692,28 @@
         <f>IF(E36="","",D36*E36)</f>
         <v/>
       </c>
+      <c r="G36" s="13" t="n"/>
+      <c r="H36" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="13" t="n">
+      <c r="A37" s="15" t="n">
         <v>32</v>
       </c>
-      <c r="B37" s="14" t="inlineStr">
+      <c r="B37" s="16" t="inlineStr">
         <is>
           <t>EVERY DAY TEA WHITENER 2KG 1 POUCH</t>
         </is>
       </c>
-      <c r="C37" s="15" t="inlineStr">
+      <c r="C37" s="17" t="inlineStr">
         <is>
           <t>PKT</t>
         </is>
       </c>
-      <c r="D37" s="16" t="n">
+      <c r="D37" s="18" t="n">
         <v>260</v>
       </c>
       <c r="E37" s="11" t="n"/>
@@ -1431,6 +1721,12 @@
         <f>IF(E37="","",D37*E37)</f>
         <v/>
       </c>
+      <c r="G37" s="19" t="n"/>
+      <c r="H37" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="7" t="n">
@@ -1454,22 +1750,28 @@
         <f>IF(E38="","",D38*E38)</f>
         <v/>
       </c>
+      <c r="G38" s="13" t="n"/>
+      <c r="H38" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="13" t="n">
+      <c r="A39" s="15" t="n">
         <v>34</v>
       </c>
-      <c r="B39" s="14" t="inlineStr">
+      <c r="B39" s="16" t="inlineStr">
         <is>
           <t>LIPTON TEA BAG 600 BAGS</t>
         </is>
       </c>
-      <c r="C39" s="15" t="inlineStr">
+      <c r="C39" s="17" t="inlineStr">
         <is>
           <t>BOX</t>
         </is>
       </c>
-      <c r="D39" s="16" t="n">
+      <c r="D39" s="18" t="n">
         <v>10</v>
       </c>
       <c r="E39" s="11" t="n"/>
@@ -1477,6 +1779,12 @@
         <f>IF(E39="","",D39*E39)</f>
         <v/>
       </c>
+      <c r="G39" s="19" t="n"/>
+      <c r="H39" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="7" t="n">
@@ -1500,22 +1808,28 @@
         <f>IF(E40="","",D40*E40)</f>
         <v/>
       </c>
+      <c r="G40" s="13" t="n"/>
+      <c r="H40" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="13" t="n">
+      <c r="A41" s="15" t="n">
         <v>36</v>
       </c>
-      <c r="B41" s="14" t="inlineStr">
+      <c r="B41" s="16" t="inlineStr">
         <is>
           <t>NESTLE WATER 500 ML</t>
         </is>
       </c>
-      <c r="C41" s="15" t="inlineStr">
+      <c r="C41" s="17" t="inlineStr">
         <is>
           <t>CRT</t>
         </is>
       </c>
-      <c r="D41" s="16" t="n">
+      <c r="D41" s="18" t="n">
         <v>23</v>
       </c>
       <c r="E41" s="11" t="n"/>
@@ -1523,6 +1837,12 @@
         <f>IF(E41="","",D41*E41)</f>
         <v/>
       </c>
+      <c r="G41" s="19" t="n"/>
+      <c r="H41" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="7" t="n">
@@ -1546,22 +1866,28 @@
         <f>IF(E42="","",D42*E42)</f>
         <v/>
       </c>
+      <c r="G42" s="13" t="n"/>
+      <c r="H42" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="13" t="n">
+      <c r="A43" s="15" t="n">
         <v>38</v>
       </c>
-      <c r="B43" s="14" t="inlineStr">
+      <c r="B43" s="16" t="inlineStr">
         <is>
           <t>TAPAL FAMILY MIXTURE (900GM)</t>
         </is>
       </c>
-      <c r="C43" s="15" t="inlineStr">
+      <c r="C43" s="17" t="inlineStr">
         <is>
           <t>PKT</t>
         </is>
       </c>
-      <c r="D43" s="16" t="n">
+      <c r="D43" s="18" t="n">
         <v>176</v>
       </c>
       <c r="E43" s="11" t="n"/>
@@ -1569,46 +1895,189 @@
         <f>IF(E43="","",D43*E43)</f>
         <v/>
       </c>
-    </row>
-    <row r="44" ht="24" customHeight="1">
-      <c r="A44" s="17" t="inlineStr">
-        <is>
-          <t>TOTAL PURCHASED</t>
-        </is>
-      </c>
-      <c r="F44" s="18">
+      <c r="G43" s="19" t="n"/>
+      <c r="H43" s="14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="6" customHeight="1"/>
+    <row r="45" ht="24" customHeight="1">
+      <c r="A45" s="20" t="inlineStr">
+        <is>
+          <t>TOTAL PURCHASED (ALL ITEMS)</t>
+        </is>
+      </c>
+      <c r="F45" s="21">
         <f>SUM(F6:F43)</f>
         <v/>
       </c>
     </row>
-    <row r="45" ht="24" customHeight="1">
-      <c r="A45" s="19" t="inlineStr">
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  → Cash Purchases Total</t>
+        </is>
+      </c>
+      <c r="F46" s="23">
+        <f>SUMIF(H6:H43,"Cash",F6:F43)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  → Credit Purchases Total</t>
+        </is>
+      </c>
+      <c r="F47" s="25">
+        <f>SUMIF(H6:H43,"Credit",F6:F43)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="26" t="inlineStr">
         <is>
           <t>BALANCE  (Advance − Total)</t>
         </is>
       </c>
-      <c r="F45" s="20">
-        <f>IF(F3="","",F3-F44)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="21" t="inlineStr">
-        <is>
-          <t>📝  KASHIF: Sirf RATE (PKR) column fill karein — orange cells mein.  |  Hassan: Date, Customer aur Advance pehle fill karein.</t>
+      <c r="F48" s="27">
+        <f>IF(F3="","",F3-F45)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="28" t="inlineStr">
+        <is>
+          <t>ZOHO ENTRIES THAT WILL BE CREATED AUTOMATICALLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B51" s="30" t="inlineStr">
+        <is>
+          <t>Expense Entry</t>
+        </is>
+      </c>
+      <c r="D51" s="31" t="inlineStr">
+        <is>
+          <t>Advance paid to Kashif</t>
+        </is>
+      </c>
+      <c r="G51" s="32" t="inlineStr">
+        <is>
+          <t>Paid From account → Kashif Advance</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" s="29" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B52" s="33" t="inlineStr">
+        <is>
+          <t>Vendor Bills (Cash)</t>
+        </is>
+      </c>
+      <c r="D52" s="34" t="inlineStr">
+        <is>
+          <t>One bill per vendor for cash items</t>
+        </is>
+      </c>
+      <c r="G52" s="35" t="inlineStr">
+        <is>
+          <t>COGS Dr / Vendor Cr (adjust vs advance)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="29" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B53" s="30" t="inlineStr">
+        <is>
+          <t>Vendor Bills (Credit)</t>
+        </is>
+      </c>
+      <c r="D53" s="31" t="inlineStr">
+        <is>
+          <t>One bill per credit vendor</t>
+        </is>
+      </c>
+      <c r="G53" s="32" t="inlineStr">
+        <is>
+          <t>COGS Dr / Accounts Payable Cr</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="29" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B54" s="33" t="inlineStr">
+        <is>
+          <t>Customer Invoice</t>
+        </is>
+      </c>
+      <c r="D54" s="34" t="inlineStr">
+        <is>
+          <t>Sales invoice for customer</t>
+        </is>
+      </c>
+      <c r="G54" s="35" t="inlineStr">
+        <is>
+          <t>Customer Receivable Dr / Sales Cr</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A47:F47"/>
+  <mergeCells count="25">
+    <mergeCell ref="B54:C54"/>
+    <mergeCell ref="A48:E48"/>
+    <mergeCell ref="G52:H52"/>
     <mergeCell ref="B3:C3"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2"/>
+    <mergeCell ref="A53"/>
     <mergeCell ref="A45:E45"/>
-    <mergeCell ref="A44:E44"/>
+    <mergeCell ref="A52"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="D53:F53"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="A51"/>
+    <mergeCell ref="A46:E46"/>
+    <mergeCell ref="G53:H53"/>
+    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="A50:H50"/>
+    <mergeCell ref="D51:F51"/>
+    <mergeCell ref="D54:F54"/>
+    <mergeCell ref="A47:E47"/>
+    <mergeCell ref="A54"/>
     <mergeCell ref="D3:E3"/>
+    <mergeCell ref="G51:H51"/>
+    <mergeCell ref="G54:H54"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="D52:F52"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="G3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Petty Cash,NEW CASH APRIL ONWARD,HBL,Habib Metro Bank,Faysal Bank"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H42 H43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Cash,Credit"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToWidth="1"/>
 </worksheet>

</xml_diff>